<commit_message>
Fix: Actualizou-se o ficheiro excel 1
</commit_message>
<xml_diff>
--- a/notas.xlsx
+++ b/notas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerson B Hungulu\Documents\Desenvolvimento de Software\appWeb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A922A5D7-DF5D-472B-AA69-642B1A656787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B36AAC0-B412-4434-ACA0-0BA67BA44D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>N.º Estudante</t>
   </si>
@@ -143,13 +143,7 @@
     <t>Janeth Pereira</t>
   </si>
   <si>
-    <t>22108755</t>
-  </si>
-  <si>
     <t>José Jacunana</t>
-  </si>
-  <si>
-    <t>22119148</t>
   </si>
   <si>
     <t>João Gravino</t>
@@ -210,7 +204,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -245,8 +239,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -265,8 +271,14 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFEFEF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -300,11 +312,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -329,6 +371,24 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -732,7 +792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -745,7 +805,7 @@
     <row r="1" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:6" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>0</v>
       </c>
@@ -765,507 +825,500 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5">
+      <c r="C5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="11">
         <v>0</v>
       </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F5" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="12">
         <v>15.4</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="11">
         <v>18</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="11">
         <v>16.7</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="12">
         <v>15</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="11">
         <v>0</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="11">
         <v>7.5</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="12">
         <v>19.7</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="11">
         <v>18</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="11">
         <v>18.850000000000001</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="12">
         <v>19.8</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="11">
         <v>16</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="11">
         <v>17.899999999999999</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="12">
         <v>20</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="11">
         <v>0</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="11">
         <v>10</v>
       </c>
-      <c r="F10">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="12">
         <v>13.5</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="11">
         <v>7</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="11">
         <v>10.25</v>
       </c>
-      <c r="F11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F11" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="12">
         <v>17.100000000000001</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="11">
         <v>18</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="11">
         <v>17.55</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="12">
         <v>17.8</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="11">
         <v>0</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="11">
         <v>8.9</v>
       </c>
-      <c r="F13">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="12">
         <v>15.2</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="11">
         <v>0</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="11">
         <v>7.6</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="11">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="12">
         <v>20</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="11">
         <v>0</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="11">
         <v>10</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="11">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="12">
         <v>19.600000000000001</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="11">
         <v>18</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="11">
         <v>18.8</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="11">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="12">
         <v>16.7</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="11">
         <v>18</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="11">
         <v>17.350000000000001</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="11">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="12">
         <v>16.399999999999999</v>
       </c>
-      <c r="D18" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18">
+      <c r="D18" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="11">
         <v>8.1999999999999993</v>
       </c>
-      <c r="F18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="F18" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>22119148</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="12">
+        <v>18.5</v>
+      </c>
+      <c r="D19" s="11">
+        <v>14</v>
+      </c>
+      <c r="E19" s="11">
+        <v>16.25</v>
+      </c>
+      <c r="F19" s="11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>22108755</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19">
-        <v>18.5</v>
-      </c>
-      <c r="D19">
+      <c r="C20" s="12">
+        <v>19.8</v>
+      </c>
+      <c r="D20" s="11">
+        <v>5</v>
+      </c>
+      <c r="E20" s="11">
+        <v>12.4</v>
+      </c>
+      <c r="F20" s="11">
         <v>14</v>
       </c>
-      <c r="E19">
-        <v>16.25</v>
-      </c>
-      <c r="F19">
+    </row>
+    <row r="21" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="12">
+        <v>19.3</v>
+      </c>
+      <c r="D21" s="11">
+        <v>16</v>
+      </c>
+      <c r="E21" s="11">
+        <v>17.649999999999999</v>
+      </c>
+      <c r="F21" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="11">
+        <v>0</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="12">
+        <v>15.7</v>
+      </c>
+      <c r="D23" s="11">
+        <v>0</v>
+      </c>
+      <c r="E23" s="11">
+        <v>7.85</v>
+      </c>
+      <c r="F23" s="11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="12">
+        <v>17</v>
+      </c>
+      <c r="D24" s="11">
+        <v>0</v>
+      </c>
+      <c r="E24" s="11">
+        <v>8.5</v>
+      </c>
+      <c r="F24" s="11">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20">
-        <v>19.8</v>
-      </c>
-      <c r="D20">
-        <v>5</v>
-      </c>
-      <c r="E20">
-        <v>12.4</v>
-      </c>
-      <c r="F20">
+    <row r="25" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="12">
+        <v>19</v>
+      </c>
+      <c r="D25" s="11">
+        <v>12</v>
+      </c>
+      <c r="E25" s="11">
+        <v>15.5</v>
+      </c>
+      <c r="F25" s="11">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21">
-        <v>19.3</v>
-      </c>
-      <c r="D21">
-        <v>16</v>
-      </c>
-      <c r="E21">
-        <v>17.649999999999999</v>
-      </c>
-      <c r="F21">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22">
+    <row r="26" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="12">
+        <v>19.2</v>
+      </c>
+      <c r="D26" s="11">
         <v>0</v>
       </c>
-      <c r="F22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23">
-        <v>15.7</v>
-      </c>
-      <c r="D23">
+      <c r="E26" s="11">
+        <v>9.6</v>
+      </c>
+      <c r="F26" s="11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="11">
         <v>0</v>
       </c>
-      <c r="E23">
-        <v>7.85</v>
-      </c>
-      <c r="F23">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24">
-        <v>17</v>
-      </c>
-      <c r="D24">
+      <c r="F27" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C28" s="12">
+        <v>20</v>
+      </c>
+      <c r="D28" s="11">
         <v>0</v>
       </c>
-      <c r="E24">
-        <v>8.5</v>
-      </c>
-      <c r="F24">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25">
-        <v>19</v>
-      </c>
-      <c r="D25">
-        <v>12</v>
-      </c>
-      <c r="E25">
-        <v>15.5</v>
-      </c>
-      <c r="F25">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26">
-        <v>19.2</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>9.6</v>
-      </c>
-      <c r="F26">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" t="s">
-        <v>8</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="E28" s="11">
+        <v>10</v>
+      </c>
+      <c r="F28" s="11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28">
-        <v>20</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>10</v>
-      </c>
-      <c r="F28">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="6" t="s">
-        <v>55</v>
       </c>
       <c r="B29" s="7">
         <f>COUNTA(A5:A28)</f>
         <v>24</v>
       </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29">
-        <v>0</v>
-      </c>
-      <c r="F29" t="s">
-        <v>8</v>
-      </c>
-    </row>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="10"/>
+    </row>
+    <row r="30" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>